<commit_message>
Budget: new month timeline (every month with in/out bars, centred on the open one); import and template handle transfers to your own accounts, pockets, brokers and exchanges
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/Trackr-transactions-template.xlsx
+++ b/templates/Trackr-transactions-template.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Lists" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Transactions!$A$1:$M$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Transactions!$A$1:$O$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3">Categories!$A$1:$C$268</definedName>
   </definedNames>
 </workbook>
@@ -408,7 +408,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:O1"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -418,11 +418,13 @@
     <col min="6" max="6" width="18.83203125" customWidth="1"/>
     <col min="7" max="7" width="15.83203125" customWidth="1"/>
     <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" customWidth="1"/>
-    <col min="10" max="10" width="9.83203125" customWidth="1"/>
-    <col min="11" max="11" width="11.83203125" customWidth="1"/>
-    <col min="12" max="12" width="14.83203125" customWidth="1"/>
-    <col min="13" max="13" width="28.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="24.83203125" customWidth="1"/>
+    <col min="11" max="11" width="15.83203125" customWidth="1"/>
+    <col min="12" max="12" width="9.83203125" customWidth="1"/>
+    <col min="13" max="13" width="11.83203125" customWidth="1"/>
+    <col min="14" max="14" width="14.83203125" customWidth="1"/>
+    <col min="15" max="15" width="28.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -451,26 +453,32 @@
         <v>Account</v>
       </c>
       <c r="I1" t="str">
+        <v>From</v>
+      </c>
+      <c r="J1" t="str">
+        <v>To</v>
+      </c>
+      <c r="K1" t="str">
         <v>Personal Impact</v>
       </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>Currency</v>
       </c>
-      <c r="K1" t="str">
+      <c r="M1" t="str">
         <v>Amount</v>
       </c>
-      <c r="L1" t="str">
+      <c r="N1" t="str">
         <v>Location</v>
       </c>
-      <c r="M1" t="str">
+      <c r="O1" t="str">
         <v>Description</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M1"/>
+  <autoFilter ref="A1:O1"/>
   <dataValidations count="7">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0" sqref="C2:C2000">
-      <formula1>Lists!$A$2:$A$3</formula1>
+      <formula1>Lists!$A$2:$A$4</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0" sqref="D2:D2000">
       <formula1>OFFSET(Lists!$G$2,0,IF($C2="Income",1,0),IF($C2="Income",12,20),1)</formula1>
@@ -481,10 +489,10 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0" sqref="F2:F2000">
       <formula1>Lists!$C$2:$C$3</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0" sqref="I2:I2000">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0" sqref="K2:K2000">
       <formula1>Lists!$D$2:$D$4</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0" sqref="J2:J2000">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0" sqref="L2:L2000">
       <formula1>Lists!$B$2:$B$5</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0" sqref="G2:G2000">
@@ -492,14 +500,14 @@
     </dataValidation>
   </dataValidations>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A32"/>
   <cols>
     <col min="1" max="1" width="130.83203125" customWidth="1"/>
   </cols>
@@ -521,7 +529,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2. Only Date and Amount are required. Type, Category, Sub-category, Recurring, Payment Method, Account, Personal Impact and Currency have drop-down lists (in Excel).</v>
+        <v>2. Only Date and Amount are required. Type, Category, Sub-category, Recurring, Payment Method, Account, From, To, Personal Impact and Currency have drop-down lists (in Excel).</v>
       </c>
     </row>
     <row r="5">
@@ -556,7 +564,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>• Type — Expense or Income. Leave empty to use the sign of Amount (negative = expense).</v>
+        <v>• Type — Expense, Income or Transfer (money moving between your own accounts, pockets, brokers or exchanges — then fill From and To). Leave empty to use the sign of Amount (negative = expense).</v>
       </c>
     </row>
     <row r="12">
@@ -581,84 +589,99 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>• Account — Optional — one of your bank accounts in Trackr (from the list).</v>
+        <v>• Account — Optional — one of your bank accounts in Trackr (from the list). Not used for a transfer (see From / To).</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>• Personal Impact — Optional — Neutral, Positive or Negative.</v>
+        <v>• From — Transfers only — where the money leaves: a bank account, a pocket ("Account › Pocket"), a broker or an exchange (from the list).</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>• Currency — EUR, USD, GBP or CHF. Empty = the account's currency, otherwise your default one.</v>
+        <v>• To — Transfers only — where the money arrives (same list as From).</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>• Amount (required) — A number like 12.50. Negative is fine — with Type empty it then counts as an expense.</v>
+        <v>• Personal Impact — Optional — Neutral, Positive or Negative.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>• Location — Optional.</v>
+        <v>• Currency — EUR, USD, GBP or CHF. Empty = the account's currency, otherwise your default one.</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>• Description — Optional note.</v>
+        <v>• Amount (required) — A number like 12.50. Negative is fine — with Type empty it then counts as an expense.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v/>
+        <v>• Location — Optional.</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Tips</v>
+        <v>• Description — Optional note.</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>• See the "Example" sheet for filled-in rows, and "Categories" / "Lists" for every name Trackr knows.</v>
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>• The Category list follows the Type you picked, and the Sub-category list follows the Category. You can still type a new name — it will be created.</v>
+        <v>Tips</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>• Transfers (to a pocket, broker or exchange) can't be imported — add those in Trackr with Budget → Add transaction → Transfer.</v>
+        <v>• See the "Example" sheet for filled-in rows, and "Categories" / "Lists" for every name Trackr knows.</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>• Bank exports (Excel or CSV) usually work as they are: Date, Amount (or Debit/Credit columns) and Description are recognised, in English, French or Dutch.</v>
+        <v>• The Category list follows the Type you picked, and the Sub-category list follows the Category. You can still type a new name — it will be created.</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>• Budget → Export to Excel uses these same column names, so you can export, edit and re-import.</v>
+        <v>• Transfers: money moving between your own places — bank account → pocket, → another bank account, → a broker's or exchange's cash. Type "Transfer", then From and To (pick from the lists; a pocket is "Account › Pocket"). Category, Account and Recurring are left empty. A transfer is neither income nor spending.</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>• Account balances only change if you tick "Also update account balances" in the preview.</v>
+        <v>• In a bank export, a transfer to your own savings account or pocket is recognised from its name or its Type/Category; the preview lets you choose where it went if Trackr can't tell.</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>• Bank exports (Excel or CSV) usually work as they are: Date, Amount (or Debit/Credit columns) and Description are recognised, in English, French or Dutch.</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>• Budget → Export to Excel uses these same column names, so you can export, edit and re-import.</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>• Account balances (and pockets, broker and exchange cash for transfers) only change if you tick "Also update balances" in the preview.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A32"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:O11"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -668,11 +691,13 @@
     <col min="6" max="6" width="18.83203125" customWidth="1"/>
     <col min="7" max="7" width="15.83203125" customWidth="1"/>
     <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" customWidth="1"/>
-    <col min="10" max="10" width="9.83203125" customWidth="1"/>
-    <col min="11" max="11" width="11.83203125" customWidth="1"/>
-    <col min="12" max="12" width="14.83203125" customWidth="1"/>
-    <col min="13" max="13" width="28.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="24.83203125" customWidth="1"/>
+    <col min="11" max="11" width="15.83203125" customWidth="1"/>
+    <col min="12" max="12" width="9.83203125" customWidth="1"/>
+    <col min="13" max="13" width="11.83203125" customWidth="1"/>
+    <col min="14" max="14" width="14.83203125" customWidth="1"/>
+    <col min="15" max="15" width="28.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -701,18 +726,24 @@
         <v>Account</v>
       </c>
       <c r="I1" t="str">
+        <v>From</v>
+      </c>
+      <c r="J1" t="str">
+        <v>To</v>
+      </c>
+      <c r="K1" t="str">
         <v>Personal Impact</v>
       </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>Currency</v>
       </c>
-      <c r="K1" t="str">
+      <c r="M1" t="str">
         <v>Amount</v>
       </c>
-      <c r="L1" t="str">
+      <c r="N1" t="str">
         <v>Location</v>
       </c>
-      <c r="M1" t="str">
+      <c r="O1" t="str">
         <v>Description</v>
       </c>
     </row>
@@ -742,18 +773,24 @@
         <v/>
       </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
         <v>Neutral</v>
       </c>
-      <c r="J2" t="str">
+      <c r="L2" t="str">
         <v>EUR</v>
       </c>
-      <c r="K2" s="2">
+      <c r="M2" s="2">
         <v>850</v>
       </c>
-      <c r="L2" t="str">
-        <v/>
-      </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
         <v>Monthly pay</v>
       </c>
     </row>
@@ -783,18 +820,24 @@
         <v/>
       </c>
       <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
         <v>Neutral</v>
       </c>
-      <c r="J3" t="str">
+      <c r="L3" t="str">
         <v>EUR</v>
       </c>
-      <c r="K3" s="2">
+      <c r="M3" s="2">
         <v>450</v>
       </c>
-      <c r="L3" t="str">
-        <v/>
-      </c>
-      <c r="M3" t="str">
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
         <v/>
       </c>
     </row>
@@ -824,18 +867,24 @@
         <v/>
       </c>
       <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
         <v>Neutral</v>
       </c>
-      <c r="J4" t="str">
+      <c r="L4" t="str">
         <v>EUR</v>
       </c>
-      <c r="K4" s="2">
+      <c r="M4" s="2">
         <v>200</v>
       </c>
-      <c r="L4" t="str">
-        <v/>
-      </c>
-      <c r="M4" t="str">
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
         <v/>
       </c>
     </row>
@@ -865,18 +914,24 @@
         <v/>
       </c>
       <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
         <v>Neutral</v>
       </c>
-      <c r="J5" t="str">
+      <c r="L5" t="str">
         <v>EUR</v>
       </c>
-      <c r="K5" s="2">
+      <c r="M5" s="2">
         <v>23.4</v>
       </c>
-      <c r="L5" t="str">
+      <c r="N5" t="str">
         <v>Maastricht</v>
       </c>
-      <c r="M5" t="str">
+      <c r="O5" t="str">
         <v/>
       </c>
     </row>
@@ -906,18 +961,24 @@
         <v/>
       </c>
       <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
         <v>Neutral</v>
       </c>
-      <c r="J6" t="str">
+      <c r="L6" t="str">
         <v>EUR</v>
       </c>
-      <c r="K6" s="2">
+      <c r="M6" s="2">
         <v>6.99</v>
       </c>
-      <c r="L6" t="str">
-        <v/>
-      </c>
-      <c r="M6" t="str">
+      <c r="N6" t="str">
+        <v/>
+      </c>
+      <c r="O6" t="str">
         <v/>
       </c>
     </row>
@@ -947,18 +1008,24 @@
         <v/>
       </c>
       <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
         <v>Neutral</v>
       </c>
-      <c r="J7" t="str">
+      <c r="L7" t="str">
         <v>EUR</v>
       </c>
-      <c r="K7" s="2">
+      <c r="M7" s="2">
         <v>25.5</v>
       </c>
-      <c r="L7" t="str">
-        <v/>
-      </c>
-      <c r="M7" t="str">
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="str">
         <v>Weekend trip</v>
       </c>
     </row>
@@ -988,65 +1055,171 @@
         <v/>
       </c>
       <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
         <v>Positive</v>
       </c>
-      <c r="J8" t="str">
+      <c r="L8" t="str">
         <v>EUR</v>
       </c>
-      <c r="K8" s="2">
+      <c r="M8" s="2">
         <v>10</v>
       </c>
-      <c r="L8" t="str">
-        <v/>
-      </c>
-      <c r="M8" t="str">
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="str">
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Coffee</v>
+        <v>Holiday savings</v>
       </c>
       <c r="B9" s="1">
-        <v>46277</v>
+        <v>46267</v>
       </c>
       <c r="C9" t="str">
-        <v/>
+        <v>Transfer</v>
       </c>
       <c r="D9" t="str">
-        <v>Food &amp; Groceries</v>
+        <v/>
       </c>
       <c r="E9" t="str">
-        <v>Coffee &amp; Snacks</v>
+        <v/>
       </c>
       <c r="F9" t="str">
         <v>One-off / Variable</v>
       </c>
       <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v>Current account</v>
+      </c>
+      <c r="J9" t="str">
+        <v>Current account › Holidays</v>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
+        <v>EUR</v>
+      </c>
+      <c r="M9" s="2">
+        <v>100</v>
+      </c>
+      <c r="N9" t="str">
+        <v/>
+      </c>
+      <c r="O9" t="str">
+        <v>Into the pocket</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Monthly ETF money</v>
+      </c>
+      <c r="B10" s="1">
+        <v>46270</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Transfer</v>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v>One-off / Variable</v>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v>Current account</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Trade Republic (broker)</v>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
+        <v>EUR</v>
+      </c>
+      <c r="M10" s="2">
+        <v>50</v>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Coffee</v>
+      </c>
+      <c r="B11" s="1">
+        <v>46277</v>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v>Food &amp; Groceries</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Coffee &amp; Snacks</v>
+      </c>
+      <c r="F11" t="str">
+        <v>One-off / Variable</v>
+      </c>
+      <c r="G11" t="str">
         <v>Card</v>
       </c>
-      <c r="H9" t="str">
-        <v/>
-      </c>
-      <c r="I9" t="str">
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
         <v>Neutral</v>
       </c>
-      <c r="J9" t="str">
+      <c r="L11" t="str">
         <v>EUR</v>
       </c>
-      <c r="K9" s="2">
+      <c r="M11" s="2">
         <v>-3.2</v>
       </c>
-      <c r="L9" t="str">
-        <v/>
-      </c>
-      <c r="M9" t="str">
+      <c r="N11" t="str">
+        <v/>
+      </c>
+      <c r="O11" t="str">
         <v>Type empty + negative amount = expense</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O11"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4823,7 +4996,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:I21"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -4833,6 +5006,7 @@
     <col min="6" max="6" width="22.83203125" customWidth="1"/>
     <col min="7" max="7" width="22.83203125" customWidth="1"/>
     <col min="8" max="8" width="22.83203125" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4860,6 +5034,9 @@
       <c r="H1" t="str">
         <v>Income categories</v>
       </c>
+      <c r="I1" t="str">
+        <v>Transfer places</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -4886,6 +5063,9 @@
       <c r="H2" t="str">
         <v>Salary</v>
       </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -4912,10 +5092,13 @@
       <c r="H3" t="str">
         <v>Freelance</v>
       </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v/>
+        <v>Transfer</v>
       </c>
       <c r="B4" t="str">
         <v>GBP</v>
@@ -4938,6 +5121,9 @@
       <c r="H4" t="str">
         <v>Family Support</v>
       </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -4964,6 +5150,9 @@
       <c r="H5" t="str">
         <v>Scholarships &amp; Grants</v>
       </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -4990,6 +5179,9 @@
       <c r="H6" t="str">
         <v>Government Benefits</v>
       </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -5016,6 +5208,9 @@
       <c r="H7" t="str">
         <v>Student Loans &amp; Credit</v>
       </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -5042,6 +5237,9 @@
       <c r="H8" t="str">
         <v>Investment Returns</v>
       </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -5068,6 +5266,9 @@
       <c r="H9" t="str">
         <v>Rental Income</v>
       </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -5094,6 +5295,9 @@
       <c r="H10" t="str">
         <v>Sales &amp; Resale</v>
       </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -5120,6 +5324,9 @@
       <c r="H11" t="str">
         <v>Refunds &amp; Reimbursements</v>
       </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -5146,6 +5353,9 @@
       <c r="H12" t="str">
         <v>Gifts Received</v>
       </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -5172,6 +5382,9 @@
       <c r="H13" t="str">
         <v>Other</v>
       </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -5198,6 +5411,9 @@
       <c r="H14" t="str">
         <v/>
       </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -5224,6 +5440,9 @@
       <c r="H15" t="str">
         <v/>
       </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -5250,6 +5469,9 @@
       <c r="H16" t="str">
         <v/>
       </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -5276,6 +5498,9 @@
       <c r="H17" t="str">
         <v/>
       </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -5302,6 +5527,9 @@
       <c r="H18" t="str">
         <v/>
       </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -5328,6 +5556,9 @@
       <c r="H19" t="str">
         <v/>
       </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -5354,6 +5585,9 @@
       <c r="H20" t="str">
         <v/>
       </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -5380,10 +5614,13 @@
       <c r="H21" t="str">
         <v/>
       </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>